<commit_message>
docs: roadmap S29 marcado fechado (09/jun)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/api/sprints-pm.xlsx
+++ b/public/api/sprints-pm.xlsx
@@ -568,7 +568,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
@@ -1270,19 +1270,19 @@
           <t>0.29.0</t>
         </is>
       </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Juntar base mapping + lista de clientes sap 4 me, relatorio deve ser usual para duda ter visao de pipeline dos cases de sucesso</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
-        <is>
-          <t>⏳ A FAZER</t>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>fechado (09/jun)</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>dashboard /clientes-sap-4me + funil relatorio secao 8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: roadmap S30 fechado (09/jun)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/api/sprints-pm.xlsx
+++ b/public/api/sprints-pm.xlsx
@@ -1297,19 +1297,19 @@
           <t>0.30.0</t>
         </is>
       </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>Adicionar o processo de field marketing ao app e entender como ele pode ajudar nas datas, gerar lembretes para email marketing de deadlines e entregas</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
-        <is>
-          <t>⏳ A FAZER</t>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>fechado (09/jun)</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>tela /field-marketing + briefing template + captura ROI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: S29-S31 fechadas no roadmap + pendências atualizadas (home calendar resolvido)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/api/sprints-pm.xlsx
+++ b/public/api/sprints-pm.xlsx
@@ -1324,19 +1324,19 @@
           <t>0.31.0</t>
         </is>
       </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Remodelagem de todo workflow de conteudo - briefing -&gt; artigo -&gt; revisao SEO/GEO -&gt; publicação automática blog -&gt; capa do blog -&gt; copy redes sociais -&gt; carrossel -&gt; publicação</t>
         </is>
       </c>
-      <c r="D29" s="15" t="inlineStr">
-        <is>
-          <t>⏳ A FAZER</t>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>fechado (09/jun)</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>tela /content-pipeline + SEO/GEO checker + import redatoria (publicacao WP manual)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: v0.31.1 — calendário layers MDF+Deadlines + diagnóstico persistência D1
Calendário (/inbound/calendar):
- 2 layers novos no topo: MDF/Dev Funds (vermelho) + Deadlines de ações (rosa)
- layers reordenados por prioridade de negócio
- deadlines-2026.json: deadlines reais do email SAP Partner Marketing LAC
  (treinamento obrigatório 1º/abr · 100% EDF + 70% DDF até 1º/jul · proposals H2)

/api/version: bloco persistencia (db_path, data_dir, volume_ativo, status)
  para diagnosticar D1 (Railway volume DATA_DIR=/data).

Roadmap: S32 (calendário unificado, aguarda arquivos) + 3 pendências anotadas
  (PEND-1 validar volume · PEND-2 SSO admin consent · PEND-3 WordPress TI).

Aguardando arquivos do Rudá: planilhas Redatoria/Duda atualizadas, lista de
MDFs abertos com deadlines, ações com prazos — para popular os layers (S32).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/api/sprints-pm.xlsx
+++ b/public/api/sprints-pm.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1340,6 +1340,114 @@
         </is>
       </c>
     </row>
+    <row r="30" ht="46" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>S32</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>0.32.0</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Calendario unificado: agenda eventos + Redatoria + Duda + datas comemorativas + DEADLINES acoes + DEADLINE cada MDF aberto. Layers MDF+Deadlines criados (v0.31.1) com deadlines email SAP.</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>em andamento</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>aguarda arquivos Ruda: planilhas Redatoria/Duda + lista MDFs abertos + acoes com prazos</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="46" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>PEND-1</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>D1 Railway Volume — DATA_DIR=/data + volume montado (Ruda 09/jun). Validar persistencia entre deploys.</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>validar</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>testar: push -&gt; dados sobrevivem sem re-sync. /api/version mostra persistencia.status</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="46" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>PEND-2</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>SSO Microsoft — env vars Azure ja no Railway. Falta admin consent Graph + testar login + SSO_ENFORCE=true.</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>bloqueado humano</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Azure portal: Grant admin consent + Redirect URIs</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="46" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>PEND-3</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Publicacao WordPress automatica (S31). Pipeline entrega HTML pronto; publicar segue manual.</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>bloqueado humano</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>credenciais admin WP com TI EPI-USE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
docs: roadmap S32 (DF tracker) fechado + S33 (popular layers) criado
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/api/sprints-pm.xlsx
+++ b/public/api/sprints-pm.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1351,19 +1351,19 @@
           <t>0.32.0</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Calendario unificado: agenda eventos + Redatoria + Duda + datas comemorativas + DEADLINES acoes + DEADLINE cada MDF aberto. Layers MDF+Deadlines criados (v0.31.1) com deadlines email SAP.</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="inlineStr">
-        <is>
-          <t>em andamento</t>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Development Funds (SAP DF LAC) tracker: /development-funds com 18 proposals + 9 requests reais + budget DDF 80k + regras PDF. Derrubados (5VVWA2SLEO+66IJWEAE2B 12.1k EUR) nao somam. Deadlines de cada MDF no calendar.</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>fechado (09/jun)</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>aguarda arquivos Ruda: planilhas Redatoria/Duda + lista MDFs abertos + acoes com prazos</t>
+          <t>aprovado valido 73.8k EUR &gt; meta 56k (1jul) OK</t>
         </is>
       </c>
     </row>
@@ -1445,6 +1445,33 @@
       <c r="E33" s="3" t="inlineStr">
         <is>
           <t>credenciais admin WP com TI EPI-USE</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>S33</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>0.33.0</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Calendario: popular layers Redatoria/Duda/Deadlines acoes. Layers prontos. DF/MDF ja integrado (v0.32.0).</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
+          <t>aguarda arquivos</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Ruda: planilha Redatoria atualizada + planilha posts Duda + acoes com prazos</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: v0.34.0 — S34 Design System unificado + aposenta telas mortas + roadmap revisão
Revisão completa do app (avaliação saúde/UI-UX/dados no plano). Executado:

(1) Design System:
- public/css/office-theme.css: vars dark canônicas + utils (.kpi/.panel/.btn/.tag/.tbl/.bar/.flag)
- public/js/office-utils.js: esc/brl/fmt/fmtDate/scoreCls/expCls
- 4 telas migradas (clientes-sap-4me, field-marketing, content-pipeline,
  development-funds) removendo :root local duplicado

(2) Telas mortas aposentadas:
- dashboard + hub → redirect 301 / (substituídas por home)
- inbound/studio → segue redirect carousel · inbound/zoho-pipeline removida
- arquivos deletados, SSO returnTo/logout → /, Cmd+K limpo

(3) Roadmap S34-S37 (planilha + changelog) + mapa-fontes-dados.md atualizado
    (Zoho/SAP4ME/Field/Content/DF/Calendar)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/api/sprints-pm.xlsx
+++ b/public/api/sprints-pm.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1475,6 +1475,114 @@
         </is>
       </c>
     </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>S34</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>0.34.0</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Design System unificado: office-theme.css (vars dark canonicas + utils CSS) + office-utils.js (esc/brl/fmt). Migrar telas novas pra consumir. Elimina 14 dup :root + 12 esc().</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>a fazer</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>base de tudo</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>S35</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>0.35.0</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Refactor telas legadas pro dark: metas (light), voices, cases, painel, inbound/*. Aposentar dashboard/hub/studio/zoho-pipeline.</t>
+        </is>
+      </c>
+      <c r="D36" s="15" t="inlineStr">
+        <is>
+          <t>a fazer</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>e o que o Ruda viu</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>S36</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>0.36.0</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>Dados fechar buracos: atualizar mapa-fontes-dados.md (Zoho/SAP4ME/Field/Content/DF), etiquetar field-captura/content-corpo vazios, LinkedIn jun, health version fix.</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>a fazer</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>S37</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>0.37.0</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>server.js modularizacao: quebrar 2750 linhas em routes/ + db.js.</t>
+        </is>
+      </c>
+      <c r="D38" s="15" t="inlineStr">
+        <is>
+          <t>a fazer</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>saude long-term</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:E1"/>

</xml_diff>

<commit_message>
feat: v0.36.0 — S38 home por role/perfil + bloco Hoje + north-star strip
Home personalizada por papel: seletor 'Ver como…' com 8 personas
(Rudá/Duda/Bruna/Gui/Isabela/Marlison/Roberto/Visitante) — cada uma
reordena e filtra as seções pra mostrar primeiro o que é da pessoa.

- personas.json: email→persona (pronto pro SSO) + ordem/esconde + KPIs foco
- NORTH-STAR strip: Pipeline MKT FY R$ (Zoho) · Seguidores LinkedIn ·
  DDF aprovado válido € — 3 números grandes, sem scroll
- HOJE: posts a publicar + eventos live + claims DF expirando no dia
- MEU FOCO: 2-3 KPIs por persona com fonte etiquetada
- 16 KPI defs, todas em APIs existentes — zero endpoint novo, dado 100% real
- persona persiste em localStorage (override manual sempre disponível)
- roadmap: S34/S35 fechados, S38/S39 registrados

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/api/sprints-pm.xlsx
+++ b/public/api/sprints-pm.xlsx
@@ -567,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1486,19 +1486,19 @@
           <t>0.34.0</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Design System unificado: office-theme.css (vars dark canonicas + utils CSS) + office-utils.js (esc/brl/fmt). Migrar telas novas pra consumir. Elimina 14 dup :root + 12 esc().</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
-        <is>
-          <t>a fazer</t>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>fechado (09/jun)</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>base de tudo</t>
+          <t>office-theme.css + office-utils.js + 4 telas migradas + mortas aposentadas</t>
         </is>
       </c>
     </row>
@@ -1513,19 +1513,19 @@
           <t>0.35.0</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>Refactor telas legadas pro dark: metas (light), voices, cases, painel, inbound/*. Aposentar dashboard/hub/studio/zoho-pipeline.</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
-        <is>
-          <t>a fazer</t>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>fechado (09/jun)</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>e o que o Ruda viu</t>
+          <t>tipografia unificada: Press Start 2P so no game; titulos Inter 800, numeros JetBrains Mono</t>
         </is>
       </c>
     </row>
@@ -1580,6 +1580,60 @@
       <c r="E38" s="3" t="inlineStr">
         <is>
           <t>saude long-term</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="44" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>S38</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>0.36.0</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>Home por role/perfil: seletor Ver como... (7 personas team.json) reordena home por papel + bloco Hoje + north-star strip. personas.json pronto pro SSO.</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>a fazer</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="44" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>S39</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>0.37.0</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>/api/freshness + chips stale automaticos (Regra 7) + cards de acao com botao + teste mobile 390px.</t>
+        </is>
+      </c>
+      <c r="D40" s="15" t="inlineStr">
+        <is>
+          <t>a fazer</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: roadmap S38 fechado (10/jun)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/api/sprints-pm.xlsx
+++ b/public/api/sprints-pm.xlsx
@@ -1594,19 +1594,19 @@
           <t>0.36.0</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Home por role/perfil: seletor Ver como... (7 personas team.json) reordena home por papel + bloco Hoje + north-star strip. personas.json pronto pro SSO.</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
-        <is>
-          <t>a fazer</t>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>fechado (10/jun)</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>8 personas + north-star + Hoje + Meu foco · validado browser (Ruda+Isabela)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: roadmap S39 fechado (10/jun)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/api/sprints-pm.xlsx
+++ b/public/api/sprints-pm.xlsx
@@ -1621,19 +1621,19 @@
           <t>0.37.0</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>/api/freshness + chips stale automaticos (Regra 7) + cards de acao com botao + teste mobile 390px.</t>
         </is>
       </c>
-      <c r="D40" s="15" t="inlineStr">
-        <is>
-          <t>a fazer</t>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>fechado (10/jun)</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>mobile device-real pendente (grids auto-fit responsivos por construcao)</t>
         </is>
       </c>
     </row>

</xml_diff>